<commit_message>
Updated with bunching and Arrear report
</commit_message>
<xml_diff>
--- a/backend/config/methodology2/excel_data/class3_4.xlsx
+++ b/backend/config/methodology2/excel_data/class3_4.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="45" windowWidth="28695" windowHeight="12540"/>
+    <workbookView xWindow="120" yWindow="45" windowWidth="28695" windowHeight="12540" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="PayScale" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="247">
   <si>
     <t xml:space="preserve">PAY SCALES OF CLASS 3 &amp; 4  </t>
   </si>
@@ -635,9 +635,6 @@
   </si>
   <si>
     <t>36500-88700</t>
-  </si>
-  <si>
-    <t>20900-43800</t>
   </si>
   <si>
     <t>29500-62000</t>
@@ -1412,7 +1409,7 @@
         <v>10</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -1438,16 +1435,16 @@
         <v>16</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="J3" s="9" t="s">
         <v>18</v>
       </c>
       <c r="K3" s="29" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -1473,16 +1470,16 @@
         <v>24</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>26</v>
       </c>
       <c r="K4" s="29" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -1508,16 +1505,16 @@
         <v>24</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J5" s="9" t="s">
         <v>26</v>
       </c>
       <c r="K5" s="29" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -1543,16 +1540,16 @@
         <v>42</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J6" s="9" t="s">
         <v>44</v>
       </c>
       <c r="K6" s="29" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1578,16 +1575,16 @@
         <v>50</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>52</v>
       </c>
       <c r="K7" s="30" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1613,16 +1610,16 @@
         <v>50</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>52</v>
       </c>
       <c r="K8" s="30" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1636,7 +1633,7 @@
         <v>58</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>59</v>
@@ -1648,16 +1645,16 @@
         <v>61</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>63</v>
       </c>
       <c r="K9" s="30" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1683,16 +1680,16 @@
         <v>61</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>63</v>
       </c>
       <c r="K10" s="30" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="O10" s="9"/>
       <c r="P10" s="9"/>
@@ -1721,16 +1718,16 @@
         <v>74</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>76</v>
       </c>
       <c r="K11" s="30" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1741,7 +1738,7 @@
         <v>77</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>78</v>
@@ -1756,16 +1753,16 @@
         <v>74</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>76</v>
       </c>
       <c r="K12" s="30" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1776,7 +1773,7 @@
         <v>81</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>82</v>
@@ -1791,16 +1788,16 @@
         <v>74</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J13" s="9" t="s">
         <v>76</v>
       </c>
       <c r="K13" s="30" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1826,16 +1823,16 @@
         <v>74</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>76</v>
       </c>
       <c r="K14" s="30" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1861,16 +1858,16 @@
         <v>74</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>76</v>
       </c>
       <c r="K15" s="30" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1896,16 +1893,16 @@
         <v>105</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J16" s="9" t="s">
         <v>107</v>
       </c>
       <c r="K16" s="30" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1931,16 +1928,16 @@
         <v>105</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J17" s="9" t="s">
         <v>107</v>
       </c>
       <c r="K17" s="30" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1966,16 +1963,16 @@
         <v>105</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J18" s="9" t="s">
         <v>107</v>
       </c>
       <c r="K18" s="30" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -1986,7 +1983,7 @@
         <v>118</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>119</v>
@@ -2001,16 +1998,16 @@
         <v>105</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J19" s="9" t="s">
         <v>107</v>
       </c>
       <c r="K19" s="30" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2036,16 +2033,16 @@
         <v>127</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J20" s="9" t="s">
         <v>129</v>
       </c>
       <c r="K20" s="30" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="15.75" thickBot="1">
@@ -2071,16 +2068,16 @@
         <v>127</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J21" s="9" t="s">
         <v>129</v>
       </c>
       <c r="K21" s="30" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2106,16 +2103,16 @@
         <v>127</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J22" s="9" t="s">
         <v>129</v>
       </c>
       <c r="K22" s="30" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15.75" thickBot="1">
@@ -2129,10 +2126,10 @@
         <v>141</v>
       </c>
       <c r="D23" s="32" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>139</v>
@@ -2141,16 +2138,16 @@
         <v>127</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J23" s="9" t="s">
         <v>129</v>
       </c>
       <c r="K23" s="30" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2176,16 +2173,16 @@
         <v>127</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J24" s="9" t="s">
         <v>129</v>
       </c>
       <c r="K24" s="30" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="15.75" thickBot="1">
@@ -2211,16 +2208,16 @@
         <v>127</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J25" s="9" t="s">
         <v>129</v>
       </c>
       <c r="K25" s="30" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="15.75" thickBot="1">
@@ -2246,16 +2243,16 @@
         <v>154</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J26" s="9" t="s">
         <v>156</v>
       </c>
       <c r="K26" s="30" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="15.75" thickBot="1">
@@ -2263,13 +2260,13 @@
         <v>25</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C27" s="20" t="s">
         <v>150</v>
       </c>
       <c r="D27" s="32" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>157</v>
@@ -2281,16 +2278,16 @@
         <v>154</v>
       </c>
       <c r="H27" s="24" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J27" s="9" t="s">
         <v>156</v>
       </c>
       <c r="K27" s="30" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2316,16 +2313,16 @@
         <v>154</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J28" s="9" t="s">
         <v>156</v>
       </c>
       <c r="K28" s="30" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2351,16 +2348,16 @@
         <v>154</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J29" s="9" t="s">
         <v>156</v>
       </c>
       <c r="K29" s="30" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="15.75" thickBot="1">
@@ -2386,16 +2383,16 @@
         <v>173</v>
       </c>
       <c r="H30" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="I30" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="I30" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="J30" s="9" t="s">
         <v>175</v>
       </c>
       <c r="K30" s="30" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2421,16 +2418,16 @@
         <v>173</v>
       </c>
       <c r="H31" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="I31" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="I31" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="J31" s="9" t="s">
         <v>175</v>
       </c>
       <c r="K31" s="30" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2456,16 +2453,16 @@
         <v>173</v>
       </c>
       <c r="H32" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="I32" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="I32" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="J32" s="9" t="s">
         <v>175</v>
       </c>
       <c r="K32" s="30" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="15.75" thickBot="1">
@@ -2491,16 +2488,16 @@
         <v>173</v>
       </c>
       <c r="H33" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="I33" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="I33" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="J33" s="9" t="s">
         <v>175</v>
       </c>
       <c r="K33" s="30" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2526,16 +2523,16 @@
         <v>173</v>
       </c>
       <c r="H34" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="I34" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="J34" s="9" t="s">
         <v>175</v>
       </c>
       <c r="K34" s="30" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -3130,7 +3127,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="35" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -4407,7 +4404,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="35" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -4425,7 +4422,7 @@
         <v>193</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>197</v>
@@ -4460,34 +4457,34 @@
         <v>194</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="J3" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>214</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:11">

</xml_diff>